<commit_message>
Add event details for bonus stamp opportunities to the QR code spreadsheet
Update `exports/generate_qr_sheet.py` to append 5 new event rows to the `atlanta-passport-qr-codes.xlsx` spreadsheet, each with a unique QR code and the event name prepended to the venue in the 'Spot' column.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 91d140a3-4db3-4194-97ae-e780cbea9f09
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 25dfd73e-3eda-4367-9070-37cedf48f59b
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/fb9954b1-03a2-4563-bd46-f2c651216b72/91d140a3-4db3-4194-97ae-e780cbea9f09/VljI0U2
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/exports/atlanta-passport-qr-codes.xlsx
+++ b/exports/atlanta-passport-qr-codes.xlsx
@@ -506,6 +506,131 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="1047750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="1047750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="1047750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="1047750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="1047750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -938,7 +1063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1359,6 +1484,176 @@
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="9" t="inlineStr"/>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Battle of the Bands
+Atlantucky Brewing</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Castleberry Hill</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Bonus stamp toward your rewards total. June 13, 2026.</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>https://fb9954b1-03a2-4563-bd46-f2c651216b72-00-1zry9jh1hlhz4.kirk.replit.dev/stamp/event-battle-of-the-bands</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="4" t="inlineStr"/>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Video Game Prelims + Soccer Tourney
+Atlantucky Brewing</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Castleberry Hill</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Bonus stamp toward your rewards total. June 16, 2026.</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>https://fb9954b1-03a2-4563-bd46-f2c651216b72-00-1zry9jh1hlhz4.kirk.replit.dev/stamp/event-video-game-prelims</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="9" t="inlineStr"/>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Hot Sauce Market
+Atlantucky Brewing</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Castleberry Hill</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Bonus stamp toward your rewards total. June 20, 2026.</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>https://fb9954b1-03a2-4563-bd46-f2c651216b72-00-1zry9jh1hlhz4.kirk.replit.dev/stamp/event-hot-sauce-market</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="4" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Post-Match Vibes at Atlantucky
+Atlantucky Brewing</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Castleberry Hill</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Bonus stamp toward your rewards total. June 21, 2026.</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>https://fb9954b1-03a2-4563-bd46-f2c651216b72-00-1zry9jh1hlhz4.kirk.replit.dev/stamp/event-post-match-atlantucky</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="9" t="inlineStr"/>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Soccer Video Game Tournament + Wing Eating Comp
+Atlantucky Brewing</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Castleberry Hill</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Bonus stamp toward your rewards total. June 22–23, 2026.</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>https://fb9954b1-03a2-4563-bd46-f2c651216b72-00-1zry9jh1hlhz4.kirk.replit.dev/stamp/event-soccer-gaming-finals</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
@@ -1381,9 +1676,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Remove added event rows from the main spreadsheet
Remove the code that appended bonus stamp events as separate rows to the main "Stamp QR Codes" sheet in `generate_qr_sheet.py`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 91d140a3-4db3-4194-97ae-e780cbea9f09
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8d8096ea-2063-470f-9c91-6e0a2c28b4bb
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/fb9954b1-03a2-4563-bd46-f2c651216b72/91d140a3-4db3-4194-97ae-e780cbea9f09/VljI0U2
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/exports/atlanta-passport-qr-codes.xlsx
+++ b/exports/atlanta-passport-qr-codes.xlsx
@@ -516,131 +516,6 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>15</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1047750" cy="1047750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>16</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1047750" cy="1047750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1047750" cy="1047750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>18</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1047750" cy="1047750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>19</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1047750" cy="1047750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1063,7 +938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1484,176 +1359,6 @@
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="90" customHeight="1">
-      <c r="A16" s="9" t="inlineStr"/>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Battle of the Bands
-Atlantucky Brewing</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Castleberry Hill</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>Bonus stamp toward your rewards total. June 13, 2026.</t>
-        </is>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>https://fb9954b1-03a2-4563-bd46-f2c651216b72-00-1zry9jh1hlhz4.kirk.replit.dev/stamp/event-battle-of-the-bands</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="4" t="inlineStr"/>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Video Game Prelims + Soccer Tourney
-Atlantucky Brewing</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Castleberry Hill</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Bonus stamp toward your rewards total. June 16, 2026.</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>https://fb9954b1-03a2-4563-bd46-f2c651216b72-00-1zry9jh1hlhz4.kirk.replit.dev/stamp/event-video-game-prelims</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="9" t="inlineStr"/>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Hot Sauce Market
-Atlantucky Brewing</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Castleberry Hill</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>Bonus stamp toward your rewards total. June 20, 2026.</t>
-        </is>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>https://fb9954b1-03a2-4563-bd46-f2c651216b72-00-1zry9jh1hlhz4.kirk.replit.dev/stamp/event-hot-sauce-market</t>
-        </is>
-      </c>
-      <c r="G18" s="13" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="4" t="inlineStr"/>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Post-Match Vibes at Atlantucky
-Atlantucky Brewing</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Castleberry Hill</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Bonus stamp toward your rewards total. June 21, 2026.</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>https://fb9954b1-03a2-4563-bd46-f2c651216b72-00-1zry9jh1hlhz4.kirk.replit.dev/stamp/event-post-match-atlantucky</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="9" t="inlineStr"/>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Soccer Video Game Tournament + Wing Eating Comp
-Atlantucky Brewing</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Castleberry Hill</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>Bonus stamp toward your rewards total. June 22–23, 2026.</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>https://fb9954b1-03a2-4563-bd46-f2c651216b72-00-1zry9jh1hlhz4.kirk.replit.dev/stamp/event-soccer-gaming-finals</t>
-        </is>
-      </c>
-      <c r="G20" s="13" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
@@ -1676,14 +1381,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
 </worksheet>
 </file>
 

</xml_diff>